<commit_message>
feat: add desktop packaging scripts, icons, and cross-platform build support for WorkPulse
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -227,8 +227,14 @@
       <color rgb="0092400E"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E40AF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="39">
+  <fills count="40">
     <fill>
       <patternFill/>
     </fill>
@@ -455,6 +461,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FEF3C7"/>
         <bgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+        <bgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -770,7 +782,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -818,6 +830,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="38" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="39" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="39" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1468,134 +1486,134 @@
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>WO-261003</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>2026-10-03</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Saturday)</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Saturday</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G4" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H4" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I4" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J4" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K4" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L4" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M4" s="13" t="inlineStr">
+      <c r="G4" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I4" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J4" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K4" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L4" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
         <is>
           <t>2026-10-16 19:38:02</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>WO-261004</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Sunday)</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Sunday</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G5" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H5" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J5" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K5" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L5" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M5" s="13" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K5" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L5" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M5" s="17" t="inlineStr">
         <is>
           <t>2026-10-15 22:12:05</t>
         </is>
@@ -2027,134 +2045,134 @@
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>WO-261010</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>2026-10-10</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Saturday)</t>
         </is>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="E11" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Saturday</t>
         </is>
       </c>
-      <c r="F11" s="13" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G11" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H11" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I11" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J11" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K11" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L11" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M11" s="13" t="inlineStr">
+      <c r="G11" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H11" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J11" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K11" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L11" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M11" s="17" t="inlineStr">
         <is>
           <t>2026-10-16 19:38:02</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>WO-261011</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Sunday)</t>
         </is>
       </c>
-      <c r="E12" s="14" t="inlineStr">
+      <c r="E12" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Sunday</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="F12" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H12" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I12" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J12" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K12" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L12" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M12" s="13" t="inlineStr">
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I12" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J12" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K12" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L12" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
         <is>
           <t>2026-10-15 22:12:05</t>
         </is>
@@ -2564,134 +2582,134 @@
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>WO-261017</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Saturday)</t>
         </is>
       </c>
-      <c r="E18" s="14" t="inlineStr">
+      <c r="E18" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Saturday</t>
         </is>
       </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="F18" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G18" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H18" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I18" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J18" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K18" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L18" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M18" s="13" t="inlineStr">
+      <c r="G18" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I18" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J18" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L18" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
         <is>
           <t>2026-10-16 19:38:02</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>WO-261018</t>
         </is>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Sunday)</t>
         </is>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E19" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Sunday</t>
         </is>
       </c>
-      <c r="F19" s="13" t="inlineStr">
+      <c r="F19" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G19" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H19" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I19" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J19" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K19" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L19" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M19" s="13" t="inlineStr">
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H19" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I19" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L19" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M19" s="17" t="inlineStr">
         <is>
           <t>2026-10-15 22:12:05</t>
         </is>
@@ -2765,201 +2783,201 @@
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>WO-261024</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Saturday)</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Saturday</t>
         </is>
       </c>
-      <c r="F21" s="13" t="inlineStr">
+      <c r="F21" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G21" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H21" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I21" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J21" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K21" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L21" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M21" s="13" t="inlineStr">
+      <c r="G21" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H21" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I21" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J21" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L21" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M21" s="17" t="inlineStr">
         <is>
           <t>2026-10-16 19:38:02</t>
         </is>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>WO-261025</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>2026-10-25</t>
         </is>
       </c>
-      <c r="C22" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Sunday)</t>
         </is>
       </c>
-      <c r="E22" s="14" t="inlineStr">
+      <c r="E22" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Sunday</t>
         </is>
       </c>
-      <c r="F22" s="13" t="inlineStr">
+      <c r="F22" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G22" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H22" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I22" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J22" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K22" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L22" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M22" s="13" t="inlineStr">
+      <c r="G22" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I22" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J22" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L22" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M22" s="17" t="inlineStr">
         <is>
           <t>2026-10-15 22:12:05</t>
         </is>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>WO-261031</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>2026-10-31</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Saturday)</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E23" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Saturday</t>
         </is>
       </c>
-      <c r="F23" s="13" t="inlineStr">
+      <c r="F23" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G23" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H23" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I23" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J23" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K23" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L23" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M23" s="13" t="inlineStr">
+      <c r="G23" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H23" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I23" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J23" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L23" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M23" s="17" t="inlineStr">
         <is>
           <t>2026-10-16 19:38:02</t>
         </is>
@@ -3063,130 +3081,130 @@
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>WO-261101</t>
         </is>
       </c>
-      <c r="B2" s="13" t="n">
+      <c r="B2" s="17" t="n">
         <v>46327</v>
       </c>
-      <c r="C2" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="C2" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Sunday)</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
+      <c r="E2" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Sunday</t>
         </is>
       </c>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="F2" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G2" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H2" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I2" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J2" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K2" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L2" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M2" s="13" t="inlineStr">
+      <c r="G2" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H2" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I2" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L2" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M2" s="17" t="inlineStr">
         <is>
           <t>2026-10-15 22:12:18</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>WO-261107</t>
         </is>
       </c>
-      <c r="B3" s="13" t="n">
+      <c r="B3" s="17" t="n">
         <v>46333</v>
       </c>
-      <c r="C3" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="C3" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D3" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Saturday)</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Saturday</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="F3" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G3" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H3" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I3" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K3" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L3" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M3" s="13" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H3" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I3" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J3" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K3" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L3" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M3" s="17" t="inlineStr">
         <is>
           <t>2026-10-16 19:43:49</t>
         </is>
@@ -3390,268 +3408,268 @@
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>WO-261114</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>2026-11-14</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Saturday)</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Saturday</t>
         </is>
       </c>
-      <c r="F7" s="13" t="inlineStr">
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G7" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H7" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I7" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J7" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K7" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L7" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M7" s="13" t="inlineStr">
+      <c r="G7" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H7" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L7" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M7" s="17" t="inlineStr">
         <is>
           <t>2026-10-16 19:43:49</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>WO-261115</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>2026-11-15</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Sunday)</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Sunday</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="F8" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G8" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H8" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I8" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J8" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K8" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L8" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M8" s="13" t="inlineStr">
+      <c r="G8" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I8" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
         <is>
           <t>2026-10-15 22:12:18</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>WO-261121</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>2026-11-21</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Saturday)</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Saturday</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G9" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L9" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M9" s="13" t="inlineStr">
+      <c r="G9" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J9" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K9" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L9" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M9" s="17" t="inlineStr">
         <is>
           <t>2026-10-16 19:43:49</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>WO-261122</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>2026-11-22</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Sunday)</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E10" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Sunday</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H10" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I10" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J10" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K10" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L10" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M10" s="13" t="inlineStr">
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I10" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
         <is>
           <t>2026-10-15 22:12:18</t>
         </is>
@@ -3725,134 +3743,134 @@
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>WO-261128</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>2026-11-28</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Saturday)</t>
         </is>
       </c>
-      <c r="E12" s="14" t="inlineStr">
+      <c r="E12" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Saturday</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="F12" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H12" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I12" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J12" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K12" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L12" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M12" s="13" t="inlineStr">
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I12" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J12" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K12" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L12" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
         <is>
           <t>2026-10-16 19:43:49</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>WO-261129</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>2026-11-29</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Sunday)</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E13" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Sunday</t>
         </is>
       </c>
-      <c r="F13" s="13" t="inlineStr">
+      <c r="F13" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G13" s="13" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I13" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J13" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K13" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L13" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M13" s="13" t="inlineStr">
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H13" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I13" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J13" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K13" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L13" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M13" s="17" t="inlineStr">
         <is>
           <t>2026-10-15 22:12:18</t>
         </is>

</xml_diff>

<commit_message>
feat: add real-time Google Sheets cloud synchronization and update APK build configuration
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1250,7 +1250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.1"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2917,73 +2917,135 @@
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>WU-261028-011516</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Afro Cargo &amp; Logistics</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>adasd</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>asdad</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H23" s="12" t="n"/>
+      <c r="I23" s="11" t="inlineStr">
+        <is>
+          <t>10:30 AM</t>
+        </is>
+      </c>
+      <c r="J23" s="11" t="inlineStr">
+        <is>
+          <t>07:30 PM</t>
+        </is>
+      </c>
+      <c r="K23" s="11" t="inlineStr">
+        <is>
+          <t>02:15 PM - 03:00 PM</t>
+        </is>
+      </c>
+      <c r="L23" s="11" t="inlineStr">
+        <is>
+          <t>05:30 PM - 05:45 PM</t>
+        </is>
+      </c>
+      <c r="M23" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28 01:15:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>WO-261031</t>
         </is>
       </c>
-      <c r="B23" s="17" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>2026-10-31</t>
         </is>
       </c>
-      <c r="C23" s="18" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr">
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
         <is>
           <t>Weekly Off (Saturday)</t>
         </is>
       </c>
-      <c r="E23" s="18" t="inlineStr">
+      <c r="E24" s="18" t="inlineStr">
         <is>
           <t>Weekend / Weekly Off: Saturday</t>
         </is>
       </c>
-      <c r="F23" s="17" t="inlineStr">
+      <c r="F24" s="17" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G23" s="17" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="H23" s="18" t="inlineStr">
-        <is>
-          <t>Weekly Off</t>
-        </is>
-      </c>
-      <c r="I23" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J23" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K23" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L23" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M23" s="17" t="inlineStr">
+      <c r="G24" s="17" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>Weekly Off</t>
+        </is>
+      </c>
+      <c r="I24" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L24" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M24" s="17" t="inlineStr">
         <is>
           <t>2026-10-16 19:38:02</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="24" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>